<commit_message>
Add AI Audit Log
</commit_message>
<xml_diff>
--- a/AI_AuditLog/AI_AuditLog_Lius.xlsx
+++ b/AI_AuditLog/AI_AuditLog_Lius.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PRO192_Group1_SE203561_LyTuanKiet_Summit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Steam_Block_Layout\AI_AuditLog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B72A8A-CDA2-4F81-AC52-262800067EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F865A7-CCC7-4BFA-A59C-87B6E635AC67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Detailed Audit Log" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="91">
   <si>
     <t>DETAILED AI AUDIT LOG</t>
   </si>
@@ -377,13 +377,500 @@
   </si>
   <si>
     <t>Hiệu chỉnh lại prompt bằng lệnh bắt buộc (Override). Yêu cầu AI hủy bỏ logic responsive và thiết lập lại toàn bộ nội dung biên bản sang hướng phát triển Multi-version Static Layout.</t>
+  </si>
+  <si>
+    <t>Tháng 07</t>
+  </si>
+  <si>
+    <t>Tháng 08</t>
+  </si>
+  <si>
+    <t>Prompt Engineering / Cost Optimization</t>
+  </si>
+  <si>
+    <t>Cần tối ưu hóa câu lệnh bằng tiếng Anh chuẩn kỹ thuật để giao task cho DeepSeek, đồng thời cần dự toán lượng token/chi phí tiêu thụ để tránh lãng phí khi xử lý khối lượng file lớn.</t>
+  </si>
+  <si>
+    <t>Dịch yêu cầu sửa UI Header/Footer sang tiếng Anh ngắn gọn. Đánh giá số lượng token tiêu tốn nếu gửi file HTML 1.2k dòng và CSS 2.6k dòng lên hệ thống để refactor.</t>
+  </si>
+  <si>
+    <t>Khởi tạo prompt tiếng Anh với các từ khóa chuyên ngành, chia gạch đầu dòng rõ ràng. Phân tích chi tiết ước tính input/output token (khoảng 75k - 94k) và dự toán chi phí rất thấp (dưới 1000 VNĐ).</t>
+  </si>
+  <si>
+    <r>
+      <t>Kept:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Sử dụng toàn bộ các prompt tiếng Anh chuẩn kỹ thuật và số liệu ước tính. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Changed:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Gộp tất cả các prompt vào một file </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> duy nhất để quản lý tập trung thay vì gửi lẻ tẻ nhiều lần. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Reflection:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Sử dụng tiếng Anh với các từ khóa chuẩn (BEM, DOM, refactor) giúp AI khoanh vùng vấn đề nhanh hơn, giảm thiểu lượng reasoning token thừa.</t>
+    </r>
+  </si>
+  <si>
+    <t>Problem-Solving / Generation</t>
+  </si>
+  <si>
+    <t>UI Implementation / HTML &amp; CSS Coding</t>
+  </si>
+  <si>
+    <t>Code giao diện Steam Login tĩnh bị một số lỗi hiển thị: file HTML không nhận diện được file CSS, Header thiếu nút Install Steam và sub-nav Browse, Footer sai layout và căn lề.</t>
+  </si>
+  <si>
+    <t>Dựa vào cấu trúc UI Steam gốc và kết quả code hiện tại, hãy fix lỗi UI: thêm nút, chỉnh active state, thêm thanh Browse, fix layout Footer, và sửa lỗi đường dẫn liên kết file CSS.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Phân tích cấu trúc thư mục từ code, phát hiện lỗi đường dẫn (chỉ ra cách dùng </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>../Style/Login.css</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>). Cung cấp các khối code HTML/CSS đã được fix để hoàn thiện Header/Footer.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Kept:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Các đoạn mã fix cấu trúc Header/Footer và cách sửa đường dẫn tương đối của file CSS. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Changed:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chỉnh sửa thủ công lại một số mã màu hex để đảm bảo độ chính xác (pixel-perfect) vì màu xanh lá AI sinh ra bị lệch tone so với Steam gốc. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Reflection:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Không bao giờ tin tưởng hoàn toàn vào mã màu UI do AI sinh ra. Kỹ sư frontend luôn phải dùng color picker để đối chiếu với bản thiết kế gốc.</t>
+    </r>
+  </si>
+  <si>
+    <t>Refactoring / Problem-Solving</t>
+  </si>
+  <si>
+    <t>Code Standardization / BEM Naming Convention</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">HTML và CSS đã chạy đúng hiển thị UI nhưng tên class/ID bị lộn xộn. Cần đổi tên toàn bộ tuân thủ nghiêm ngặt theo kiến trúc BEM đã định nghĩa trong file </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> mà không làm gãy logic.</t>
+    </r>
+  </si>
+  <si>
+    <t>Thực hiện Non-destructive refactoring. Đổi tên toàn bộ class/ID khớp với cấu trúc BEM schema cung cấp sẵn. Không được thay đổi cấu trúc DOM, không sửa CSS value, không tự ý thêm bớt logic.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quét toàn bộ ~3.8k dòng code, ánh xạ (map) thành công tên class cũ sang tên class chuẩn BEM (vd: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>.header-nav__page</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>.login-form__username</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>), trả về bản HTML/CSS đồng bộ.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Kept:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Áp dụng toàn bộ hệ thống class BEM mới do AI trả về. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Changed:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Không có. Kết quả map class hoàn hảo, UI không bị vỡ. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Reflection:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Cung cấp Context Schema (cây thư mục Markdown) là phương pháp tốt nhất để ràng buộc AI làm theo đúng quy chuẩn kiến trúc của dự án, thay vì để AI tự sáng tạo tên.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Khi xử lý lỗi HTML không nhận CSS, ban đầu AI giả định rằng file CSS và HTML nằm cùng cấp thư mục, đề xuất sử dụng đường dẫn </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>./Login.css</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> hoặc cấu trúc thẻ link mặc định.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cấu trúc cây thư mục thực tế (được cung cấp qua ảnh VS Code) cho thấy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Login.html</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> nằm trong thư mục </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Web</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, còn </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Login.css</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> nằm trong thư mục </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Style</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Cross-check lỗi hiển thị trên trình duyệt (F12 Network tab báo lỗi 404 Not Found cho file CSS) và đối chiếu với cây thư mục Explorer của VS Code.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cung cấp rõ ràng cấu trúc thư mục. Sau đó, AI đã nhận diện đúng và sửa lại thành </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>../Style/Login.css</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Over-optimization / System Architecture Assumption</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Trong quá trình xử lý code Header/Footer và refactor BEM, AI tự động thêm các khối </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>@media query</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> vào file CSS với lý do giúp giao diện thân thiện với thiết bị di động (Responsive).</t>
+    </r>
+  </si>
+  <si>
+    <t>Project Requirement yêu cầu xây dựng 2 bản tĩnh (Static HTML/CSS) hoàn toàn độc lập cho Desktop và Mobile. Việc tự ý chèn logic CSS Responsive vào bản Desktop là vi phạm cấu trúc hệ thống đã chốt.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tiến hành Code Review (kiểm tra chéo) đoạn output do AI sinh ra, phát hiện các block </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>@media (max-width: 768px)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> tự động được chèn dưới cùng của các class.</t>
+    </r>
+  </si>
+  <si>
+    <t>Gạch bỏ toàn bộ các đoạn mã responsive. Cập nhật thêm vào prompt cụm từ khóa ràng buộc (Strict Constraint): Non-destructive refactoring. Do not change logic, do not add elements or styles.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -453,8 +940,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -473,8 +972,14 @@
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -512,11 +1017,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -558,6 +1072,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -565,7 +1082,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -871,7 +1388,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="25.77734375" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -883,7 +1400,7 @@
     <col min="8" max="16384" width="8.88671875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="14.4" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -894,7 +1411,7 @@
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
     </row>
-    <row r="2" spans="1:7" ht="64.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="64.2" customHeight="1">
       <c r="A2" s="10" t="s">
         <v>37</v>
       </c>
@@ -905,7 +1422,7 @@
       <c r="F2" s="14"/>
       <c r="G2" s="14"/>
     </row>
-    <row r="3" spans="1:7" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="40.049999999999997" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>1</v>
       </c>
@@ -928,121 +1445,167 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="97.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="12">
+    <row r="4" spans="1:7" ht="15" thickBot="1">
+      <c r="A4" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+    </row>
+    <row r="5" spans="1:7" ht="97.8" thickBot="1">
+      <c r="A5" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B5" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E5" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F5" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G5" s="12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="97.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="12">
+    <row r="6" spans="1:7" ht="97.8" thickBot="1">
+      <c r="A6" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C6" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D6" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E6" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F6" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G6" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="97.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="12">
+    <row r="7" spans="1:7" ht="97.8" thickBot="1">
+      <c r="A7" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B7" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C7" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D7" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E7" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G7" s="12" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="12"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="12"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="12"/>
-    </row>
-    <row r="9" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="12"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="12"/>
-    </row>
-    <row r="10" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="12"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="12"/>
-    </row>
-    <row r="11" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="12"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12"/>
-    </row>
-    <row r="12" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
+      <c r="A8" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+    </row>
+    <row r="9" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
+      <c r="A9" s="6">
+        <v>4</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
+      <c r="A10" s="6">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
+      <c r="A11" s="6">
+        <v>6</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1051,7 +1614,7 @@
       <c r="F12" s="6"/>
       <c r="G12" s="5"/>
     </row>
-    <row r="13" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -1060,7 +1623,7 @@
       <c r="F13" s="6"/>
       <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1069,7 +1632,7 @@
       <c r="F14" s="6"/>
       <c r="G14" s="5"/>
     </row>
-    <row r="15" spans="1:7" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="79.95" customHeight="1" thickBot="1">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1078,7 +1641,7 @@
       <c r="F15" s="6"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="79.95" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1087,7 +1650,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="79.95" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -1096,7 +1659,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
     </row>
-    <row r="18" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="79.95" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -1105,7 +1668,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
     </row>
-    <row r="19" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="79.95" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1114,7 +1677,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="79.95" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1123,7 +1686,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
     </row>
-    <row r="21" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="79.95" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1132,7 +1695,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
     </row>
-    <row r="22" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="79.95" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1141,7 +1704,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
     </row>
-    <row r="23" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="79.95" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1150,7 +1713,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="79.95" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1159,7 +1722,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="79.95" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1168,7 +1731,7 @@
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="1:7" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="79.95" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1178,6 +1741,10 @@
       <c r="G26" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A8:G8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1186,7 +1753,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="38.109375" bestFit="1" customWidth="1"/>
@@ -1196,26 +1763,26 @@
     <col min="6" max="6" width="51.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="15"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-    </row>
-    <row r="3" spans="1:6" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+    </row>
+    <row r="3" spans="1:6" ht="43.8" thickBot="1">
+      <c r="A3" s="15" t="s">
         <v>57</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1234,7 +1801,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="55.8" thickBot="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -1254,7 +1821,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="55.8" thickBot="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -1274,23 +1841,47 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-    </row>
-    <row r="7" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-    </row>
-    <row r="8" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="55.8" thickBot="1">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="60" customHeight="1" thickBot="1">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="60" customHeight="1" thickBot="1">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1298,7 +1889,7 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="60" customHeight="1" thickBot="1">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1306,7 +1897,7 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="60" customHeight="1" thickBot="1">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1314,7 +1905,7 @@
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
     </row>
-    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="60" customHeight="1">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -1322,7 +1913,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="60" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -1330,7 +1921,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="60" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1338,7 +1929,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="60" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1346,7 +1937,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="60" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -1354,7 +1945,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="60" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1362,7 +1953,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="60" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -1370,7 +1961,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="60" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -1378,7 +1969,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="60" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1386,7 +1977,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="60" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1394,7 +1985,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="60" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1402,7 +1993,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="60" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1410,7 +2001,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="60" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1418,7 +2009,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="60" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1426,12 +2017,12 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="30" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="18">
       <c r="A30" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6">
       <c r="A31" s="4" t="s">
         <v>16</v>
       </c>
@@ -1442,7 +2033,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6">
       <c r="A32" s="3" t="s">
         <v>14</v>
       </c>
@@ -1453,7 +2044,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="28.8">
       <c r="A33" s="3" t="s">
         <v>21</v>
       </c>
@@ -1464,7 +2055,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3">
       <c r="A34" s="3" t="s">
         <v>24</v>
       </c>
@@ -1475,7 +2066,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" ht="28.8">
       <c r="A35" s="3" t="s">
         <v>27</v>
       </c>
@@ -1486,7 +2077,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" ht="43.2">
       <c r="A36" s="3" t="s">
         <v>30</v>
       </c>

</xml_diff>